<commit_message>
Actualización de scripts RPA, mejoras en detección y limpieza de logs
</commit_message>
<xml_diff>
--- a/reporte_patologias.xlsx
+++ b/reporte_patologias.xlsx
@@ -458,7 +458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C1"/>
+  <dimension ref="A1:C2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -477,6 +477,27 @@
           <t>patologia_detectada</t>
         </is>
       </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>60</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>ECOTOMOGRAFIA PARTES BLANDAS REGION PECTORAL DERECHA
+Hallazgos: 
+Se identifica engrosamiento y aumento de la ecogenicidad del tejido subcutáneo de la
+región pectoral derecha con aspecto de cambios inflamatorios sin imagen de colección ni
+hematoma.
+En la región retroareolar se identifica nódulo hipoecoico subareolar de bordes definidos
+Planos musculares de ecogenicidad y patrón fibrilar normal.
+Impresión: 
+Cambios inflamatorios de las partes blandas de la región pectoral derecha, a correlacionar
+con antecedentes, observándose nódulo subareolar con patrón dendritico sugestivo de
+ginecomastia.</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -511,7 +532,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3">
@@ -531,7 +552,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
@@ -542,7 +563,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>0.00%</t>
         </is>
       </c>
     </row>
@@ -554,7 +575,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-02-06 05:27:12</t>
+          <t>2026-03-10 12:49:27</t>
         </is>
       </c>
     </row>

</xml_diff>